<commit_message>
Fix XLSForm converter: normalize non-ASCII typography for Enketo compatibility
strip_html() now maps common Unicode typography (en/em-dash, curly quotes,
ellipsis, >=, minus sign, arrows, etc.) to ASCII equivalents before writing
cell values. Enketo's XML parser rejects these characters in the prolog.
Update xlsform_samples/ with clean regenerated files.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/xlsform_samples/DEMO.xlsx
+++ b/tools/xlsform_samples/DEMO.xlsx
@@ -710,7 +710,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Which of the following devices do you use regularly? (Select all that apply — choose between 1 and 4)</t>
+          <t>Which of the following devices do you use regularly? (Select all that apply -- choose between 1 and 4)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>How many years ago did you complete this degree? (This item appears only when a non-Other field is selected — demonstrating item-level visibility.)</t>
+          <t>How many years ago did you complete this degree? (This item appears only when a non-Other field is selected -- demonstrating item-level visibility.)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Please briefly describe your field. (This item appears only when 'Other' is selected — demonstrating item-level conditional display.)</t>
+          <t>Please briefly describe your field. (This item appears only when 'Other' is selected -- demonstrating item-level conditional display.)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Overall, how would you rate your experience completing {study_name}? (7-point scale — demonstrating per-item Likert override and {study_name} text substitution)</t>
+          <t>Overall, how would you rate your experience completing {study_name}? (7-point scale -- demonstrating per-item Likert override and {study_name} text substitution)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>

</xml_diff>